<commit_message>
chore: update stufe-5/organspendedetektion/feature-init-draft-PTDATA-1927 pages
</commit_message>
<xml_diff>
--- a/stufe-5/organspendedetektion/feature-init-draft-PTDATA-1927/StructureDefinition-ISiKAlkoholAbusus.xlsx
+++ b/stufe-5/organspendedetektion/feature-init-draft-PTDATA-1927/StructureDefinition-ISiKAlkoholAbusus.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$79</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2981" uniqueCount="547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3060" uniqueCount="557">
   <si>
     <t>Property</t>
   </si>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-23</t>
+    <t>2025-12-11</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1225,13 +1225,17 @@
     <t>The information determined as a result of making the observation, if the information has a simple value.</t>
   </si>
   <si>
-    <t>Bedeutung: Erfasster Wert der Observation.</t>
+    <t>**Begründung Must-Support:** Erfasster Wert der Observation.</t>
   </si>
   <si>
     <t>An observation exists to have a value, though it might not if it is in error, or if it represents a group of observations.</t>
   </si>
   <si>
-    <t>http://terminology.hl7.org/ValueSet/yes-no-unknown-not-asked</t>
+    <t xml:space="preserve">type:$this}
+</t>
+  </si>
+  <si>
+    <t>closed</t>
   </si>
   <si>
     <t xml:space="preserve">obs-7
@@ -1248,6 +1252,34 @@
   </si>
   <si>
     <t>363714003 |Interprets|</t>
+  </si>
+  <si>
+    <t>Observation.value[x]:valueCodeableConcept</t>
+  </si>
+  <si>
+    <t>valueCodeableConcept</t>
+  </si>
+  <si>
+    <t>Actual result</t>
+  </si>
+  <si>
+    <t>**Begründung Must-Support:** Viele Lebenszustände (z. B. Schwangerschaftsstatus, Alkoholabusus, Raucherstatus) werden als kategorisierte Angaben kodiert und erfordern daher ein CodeableConcept.</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/ValueSet/yes-no-unknown-not-asked</t>
+  </si>
+  <si>
+    <t>Observation.value[x]:valueDateTime</t>
+  </si>
+  <si>
+    <t>valueDateTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dateTime
+</t>
+  </si>
+  <si>
+    <t>**Begründung Must-Support:** Zeitpunktbezogene Lebenszustände (z. B. erwarteter Entbindungstermin) benötigen eine eindeutige Datumsangabe als Wert.</t>
   </si>
   <si>
     <t>Observation.dataAbsentReason</t>
@@ -2059,12 +2091,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP77"/>
+  <dimension ref="A1:AP79"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="38.30078125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="38.30078125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="19.078125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -7887,7 +7919,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
         <v>376</v>
       </c>
@@ -7952,26 +7984,26 @@
         <v>18</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>227</v>
-      </c>
-      <c r="Y49" s="2"/>
+        <v>18</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>18</v>
+      </c>
       <c r="Z49" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AB49" t="s" s="2">
         <v>381</v>
       </c>
-      <c r="AA49" t="s" s="2">
-        <v>18</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>18</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>18</v>
-      </c>
+      <c r="AC49" s="2"/>
       <c r="AD49" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AE49" t="s" s="2">
-        <v>18</v>
+        <v>382</v>
       </c>
       <c r="AF49" t="s" s="2">
         <v>376</v>
@@ -7983,7 +8015,7 @@
         <v>88</v>
       </c>
       <c r="AI49" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AJ49" t="s" s="2">
         <v>100</v>
@@ -7992,62 +8024,64 @@
         <v>18</v>
       </c>
       <c r="AL49" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AM49" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AN49" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AO49" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP49" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
-    <row r="50" hidden="true">
+    <row r="50">
       <c r="A50" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>387</v>
-      </c>
-      <c r="C50" s="2"/>
+        <v>376</v>
+      </c>
+      <c r="C50" t="s" s="2">
+        <v>389</v>
+      </c>
       <c r="D50" t="s" s="2">
         <v>18</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="G50" t="s" s="2">
         <v>88</v>
       </c>
       <c r="H50" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="I50" t="s" s="2">
         <v>18</v>
       </c>
       <c r="J50" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="K50" t="s" s="2">
         <v>236</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="O50" t="s" s="2">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>18</v>
@@ -8072,14 +8106,12 @@
         <v>18</v>
       </c>
       <c r="X50" t="s" s="2">
-        <v>146</v>
-      </c>
-      <c r="Y50" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="Y50" s="2"/>
+      <c r="Z50" t="s" s="2">
         <v>392</v>
       </c>
-      <c r="Z50" t="s" s="2">
-        <v>393</v>
-      </c>
       <c r="AA50" t="s" s="2">
         <v>18</v>
       </c>
@@ -8096,7 +8128,7 @@
         <v>18</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>76</v>
@@ -8105,7 +8137,7 @@
         <v>88</v>
       </c>
       <c r="AI50" t="s" s="2">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="AJ50" t="s" s="2">
         <v>100</v>
@@ -8114,62 +8146,64 @@
         <v>18</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>18</v>
+        <v>384</v>
       </c>
       <c r="AM50" t="s" s="2">
-        <v>187</v>
+        <v>385</v>
       </c>
       <c r="AN50" t="s" s="2">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="AO50" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP50" t="s" s="2">
-        <v>18</v>
+        <v>387</v>
       </c>
     </row>
-    <row r="51" hidden="true">
+    <row r="51">
       <c r="A51" t="s" s="2">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>396</v>
-      </c>
-      <c r="C51" s="2"/>
+        <v>376</v>
+      </c>
+      <c r="C51" t="s" s="2">
+        <v>394</v>
+      </c>
       <c r="D51" t="s" s="2">
-        <v>397</v>
+        <v>18</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H51" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="I51" t="s" s="2">
         <v>18</v>
       </c>
       <c r="J51" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>236</v>
+        <v>395</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>399</v>
+        <v>378</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="O51" t="s" s="2">
-        <v>401</v>
+        <v>380</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>18</v>
@@ -8194,13 +8228,13 @@
         <v>18</v>
       </c>
       <c r="X51" t="s" s="2">
-        <v>146</v>
+        <v>18</v>
       </c>
       <c r="Y51" t="s" s="2">
-        <v>402</v>
+        <v>18</v>
       </c>
       <c r="Z51" t="s" s="2">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="AA51" t="s" s="2">
         <v>18</v>
@@ -8218,16 +8252,16 @@
         <v>18</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>396</v>
+        <v>376</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI51" t="s" s="2">
-        <v>18</v>
+        <v>383</v>
       </c>
       <c r="AJ51" t="s" s="2">
         <v>100</v>
@@ -8236,27 +8270,27 @@
         <v>18</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>404</v>
+        <v>384</v>
       </c>
       <c r="AM51" t="s" s="2">
-        <v>405</v>
+        <v>385</v>
       </c>
       <c r="AN51" t="s" s="2">
-        <v>406</v>
+        <v>386</v>
       </c>
       <c r="AO51" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP51" t="s" s="2">
-        <v>407</v>
+        <v>387</v>
       </c>
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -8267,7 +8301,7 @@
         <v>76</v>
       </c>
       <c r="G52" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H52" t="s" s="2">
         <v>18</v>
@@ -8279,19 +8313,19 @@
         <v>18</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>409</v>
+        <v>236</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>411</v>
+        <v>399</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>412</v>
+        <v>400</v>
       </c>
       <c r="O52" t="s" s="2">
-        <v>413</v>
+        <v>401</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>18</v>
@@ -8316,13 +8350,13 @@
         <v>18</v>
       </c>
       <c r="X52" t="s" s="2">
-        <v>18</v>
+        <v>146</v>
       </c>
       <c r="Y52" t="s" s="2">
-        <v>18</v>
+        <v>402</v>
       </c>
       <c r="Z52" t="s" s="2">
-        <v>18</v>
+        <v>403</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>18</v>
@@ -8340,16 +8374,16 @@
         <v>18</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH52" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI52" t="s" s="2">
-        <v>18</v>
+        <v>404</v>
       </c>
       <c r="AJ52" t="s" s="2">
         <v>100</v>
@@ -8361,10 +8395,10 @@
         <v>18</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>414</v>
+        <v>187</v>
       </c>
       <c r="AN52" t="s" s="2">
-        <v>415</v>
+        <v>405</v>
       </c>
       <c r="AO52" t="s" s="2">
         <v>18</v>
@@ -8375,21 +8409,21 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>18</v>
+        <v>407</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G53" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H53" t="s" s="2">
         <v>18</v>
@@ -8404,15 +8438,17 @@
         <v>236</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>419</v>
-      </c>
-      <c r="O53" s="2"/>
+        <v>410</v>
+      </c>
+      <c r="O53" t="s" s="2">
+        <v>411</v>
+      </c>
       <c r="P53" t="s" s="2">
         <v>18</v>
       </c>
@@ -8436,13 +8472,13 @@
         <v>18</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="Y53" t="s" s="2">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="Z53" t="s" s="2">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>18</v>
@@ -8460,13 +8496,13 @@
         <v>18</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH53" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI53" t="s" s="2">
         <v>18</v>
@@ -8478,27 +8514,27 @@
         <v>18</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="AO53" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP53" t="s" s="2">
-        <v>425</v>
+        <v>417</v>
       </c>
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8509,7 +8545,7 @@
         <v>76</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>18</v>
@@ -8521,19 +8557,19 @@
         <v>18</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>236</v>
+        <v>419</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>427</v>
+        <v>420</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>428</v>
+        <v>421</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>429</v>
+        <v>422</v>
       </c>
       <c r="O54" t="s" s="2">
-        <v>430</v>
+        <v>423</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>18</v>
@@ -8558,13 +8594,13 @@
         <v>18</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>154</v>
+        <v>18</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>431</v>
+        <v>18</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>432</v>
+        <v>18</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>18</v>
@@ -8582,13 +8618,13 @@
         <v>18</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI54" t="s" s="2">
         <v>18</v>
@@ -8603,10 +8639,10 @@
         <v>18</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>434</v>
+        <v>425</v>
       </c>
       <c r="AO54" t="s" s="2">
         <v>18</v>
@@ -8617,10 +8653,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8643,16 +8679,16 @@
         <v>18</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>436</v>
+        <v>236</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>439</v>
+        <v>429</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
@@ -8678,13 +8714,13 @@
         <v>18</v>
       </c>
       <c r="X55" t="s" s="2">
-        <v>18</v>
+        <v>154</v>
       </c>
       <c r="Y55" t="s" s="2">
-        <v>18</v>
+        <v>430</v>
       </c>
       <c r="Z55" t="s" s="2">
-        <v>18</v>
+        <v>431</v>
       </c>
       <c r="AA55" t="s" s="2">
         <v>18</v>
@@ -8702,7 +8738,7 @@
         <v>18</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>76</v>
@@ -8720,27 +8756,27 @@
         <v>18</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>440</v>
+        <v>432</v>
       </c>
       <c r="AM55" t="s" s="2">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="AN55" t="s" s="2">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="AO55" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP55" t="s" s="2">
-        <v>443</v>
+        <v>435</v>
       </c>
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8763,18 +8799,20 @@
         <v>18</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>445</v>
+        <v>236</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>446</v>
+        <v>437</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>447</v>
+        <v>438</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="O56" s="2"/>
+        <v>439</v>
+      </c>
+      <c r="O56" t="s" s="2">
+        <v>440</v>
+      </c>
       <c r="P56" t="s" s="2">
         <v>18</v>
       </c>
@@ -8798,13 +8836,13 @@
         <v>18</v>
       </c>
       <c r="X56" t="s" s="2">
-        <v>18</v>
+        <v>154</v>
       </c>
       <c r="Y56" t="s" s="2">
-        <v>18</v>
+        <v>441</v>
       </c>
       <c r="Z56" t="s" s="2">
-        <v>18</v>
+        <v>442</v>
       </c>
       <c r="AA56" t="s" s="2">
         <v>18</v>
@@ -8822,7 +8860,7 @@
         <v>18</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>76</v>
@@ -8840,27 +8878,27 @@
         <v>18</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>449</v>
+        <v>18</v>
       </c>
       <c r="AM56" t="s" s="2">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="AN56" t="s" s="2">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="AO56" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP56" t="s" s="2">
-        <v>452</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8871,7 +8909,7 @@
         <v>76</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>18</v>
@@ -8883,20 +8921,18 @@
         <v>18</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="N57" t="s" s="2">
-        <v>457</v>
-      </c>
-      <c r="O57" t="s" s="2">
-        <v>458</v>
-      </c>
+        <v>449</v>
+      </c>
+      <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
         <v>18</v>
       </c>
@@ -8944,45 +8980,45 @@
         <v>18</v>
       </c>
       <c r="AF57" t="s" s="2">
+        <v>445</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>450</v>
+      </c>
+      <c r="AM57" t="s" s="2">
+        <v>451</v>
+      </c>
+      <c r="AN57" t="s" s="2">
+        <v>452</v>
+      </c>
+      <c r="AO57" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AP57" t="s" s="2">
         <v>453</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>18</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="AK57" t="s" s="2">
-        <v>18</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>18</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="AN57" t="s" s="2">
-        <v>461</v>
-      </c>
-      <c r="AO57" t="s" s="2">
-        <v>18</v>
-      </c>
-      <c r="AP57" t="s" s="2">
-        <v>18</v>
       </c>
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -9005,15 +9041,17 @@
         <v>18</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>102</v>
+        <v>455</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>103</v>
+        <v>456</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="N58" s="2"/>
+        <v>457</v>
+      </c>
+      <c r="N58" t="s" s="2">
+        <v>458</v>
+      </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
         <v>18</v>
@@ -9062,7 +9100,7 @@
         <v>18</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>105</v>
+        <v>454</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>76</v>
@@ -9074,25 +9112,25 @@
         <v>18</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="AK58" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AL58" t="s" s="2">
-        <v>18</v>
+        <v>459</v>
       </c>
       <c r="AM58" t="s" s="2">
-        <v>18</v>
+        <v>460</v>
       </c>
       <c r="AN58" t="s" s="2">
-        <v>106</v>
+        <v>461</v>
       </c>
       <c r="AO58" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP58" t="s" s="2">
-        <v>18</v>
+        <v>462</v>
       </c>
     </row>
     <row r="59" hidden="true">
@@ -9104,7 +9142,7 @@
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
-        <v>108</v>
+        <v>18</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s" s="2">
@@ -9123,18 +9161,20 @@
         <v>18</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>109</v>
+        <v>464</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>110</v>
+        <v>465</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>111</v>
+        <v>466</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="O59" s="2"/>
+        <v>467</v>
+      </c>
+      <c r="O59" t="s" s="2">
+        <v>468</v>
+      </c>
       <c r="P59" t="s" s="2">
         <v>18</v>
       </c>
@@ -9182,7 +9222,7 @@
         <v>18</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>116</v>
+        <v>463</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>76</v>
@@ -9194,7 +9234,7 @@
         <v>18</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>117</v>
+        <v>469</v>
       </c>
       <c r="AK59" t="s" s="2">
         <v>18</v>
@@ -9203,10 +9243,10 @@
         <v>18</v>
       </c>
       <c r="AM59" t="s" s="2">
-        <v>18</v>
+        <v>470</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>106</v>
+        <v>471</v>
       </c>
       <c r="AO59" t="s" s="2">
         <v>18</v>
@@ -9217,46 +9257,42 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
-        <v>465</v>
+        <v>18</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H60" t="s" s="2">
         <v>18</v>
       </c>
       <c r="I60" t="s" s="2">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="J60" t="s" s="2">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>466</v>
+        <v>103</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="N60" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="O60" t="s" s="2">
-        <v>194</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
         <v>18</v>
       </c>
@@ -9304,19 +9340,19 @@
         <v>18</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>468</v>
+        <v>105</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH60" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI60" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AJ60" t="s" s="2">
-        <v>117</v>
+        <v>18</v>
       </c>
       <c r="AK60" t="s" s="2">
         <v>18</v>
@@ -9328,7 +9364,7 @@
         <v>18</v>
       </c>
       <c r="AN60" t="s" s="2">
-        <v>187</v>
+        <v>106</v>
       </c>
       <c r="AO60" t="s" s="2">
         <v>18</v>
@@ -9339,21 +9375,21 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>18</v>
+        <v>108</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G61" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H61" t="s" s="2">
         <v>18</v>
@@ -9365,15 +9401,17 @@
         <v>18</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>470</v>
+        <v>109</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>471</v>
+        <v>110</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>472</v>
-      </c>
-      <c r="N61" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="N61" t="s" s="2">
+        <v>112</v>
+      </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
         <v>18</v>
@@ -9422,19 +9460,19 @@
         <v>18</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>469</v>
+        <v>116</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH61" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI61" t="s" s="2">
-        <v>473</v>
+        <v>18</v>
       </c>
       <c r="AJ61" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK61" t="s" s="2">
         <v>18</v>
@@ -9443,10 +9481,10 @@
         <v>18</v>
       </c>
       <c r="AM61" t="s" s="2">
-        <v>474</v>
+        <v>18</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>475</v>
+        <v>106</v>
       </c>
       <c r="AO61" t="s" s="2">
         <v>18</v>
@@ -9457,42 +9495,46 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
-        <v>18</v>
+        <v>475</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G62" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H62" t="s" s="2">
         <v>18</v>
       </c>
       <c r="I62" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="J62" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>470</v>
+        <v>109</v>
       </c>
       <c r="L62" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="M62" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="M62" t="s" s="2">
-        <v>478</v>
-      </c>
-      <c r="N62" s="2"/>
-      <c r="O62" s="2"/>
+      <c r="N62" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="O62" t="s" s="2">
+        <v>194</v>
+      </c>
       <c r="P62" t="s" s="2">
         <v>18</v>
       </c>
@@ -9540,19 +9582,19 @@
         <v>18</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH62" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI62" t="s" s="2">
-        <v>473</v>
+        <v>18</v>
       </c>
       <c r="AJ62" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK62" t="s" s="2">
         <v>18</v>
@@ -9561,10 +9603,10 @@
         <v>18</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>474</v>
+        <v>18</v>
       </c>
       <c r="AN62" t="s" s="2">
-        <v>479</v>
+        <v>187</v>
       </c>
       <c r="AO62" t="s" s="2">
         <v>18</v>
@@ -9575,10 +9617,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9601,7 +9643,7 @@
         <v>18</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>236</v>
+        <v>480</v>
       </c>
       <c r="L63" t="s" s="2">
         <v>481</v>
@@ -9609,12 +9651,8 @@
       <c r="M63" t="s" s="2">
         <v>482</v>
       </c>
-      <c r="N63" t="s" s="2">
-        <v>483</v>
-      </c>
-      <c r="O63" t="s" s="2">
-        <v>484</v>
-      </c>
+      <c r="N63" s="2"/>
+      <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
         <v>18</v>
       </c>
@@ -9638,13 +9676,13 @@
         <v>18</v>
       </c>
       <c r="X63" t="s" s="2">
-        <v>168</v>
+        <v>18</v>
       </c>
       <c r="Y63" t="s" s="2">
-        <v>485</v>
+        <v>18</v>
       </c>
       <c r="Z63" t="s" s="2">
-        <v>486</v>
+        <v>18</v>
       </c>
       <c r="AA63" t="s" s="2">
         <v>18</v>
@@ -9662,7 +9700,7 @@
         <v>18</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>76</v>
@@ -9671,7 +9709,7 @@
         <v>88</v>
       </c>
       <c r="AI63" t="s" s="2">
-        <v>18</v>
+        <v>483</v>
       </c>
       <c r="AJ63" t="s" s="2">
         <v>100</v>
@@ -9680,13 +9718,13 @@
         <v>18</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>487</v>
+        <v>18</v>
       </c>
       <c r="AM63" t="s" s="2">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="AN63" t="s" s="2">
-        <v>406</v>
+        <v>485</v>
       </c>
       <c r="AO63" t="s" s="2">
         <v>18</v>
@@ -9697,10 +9735,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9711,7 +9749,7 @@
         <v>76</v>
       </c>
       <c r="G64" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H64" t="s" s="2">
         <v>18</v>
@@ -9723,20 +9761,16 @@
         <v>18</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>236</v>
+        <v>480</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>491</v>
-      </c>
-      <c r="N64" t="s" s="2">
-        <v>492</v>
-      </c>
-      <c r="O64" t="s" s="2">
-        <v>493</v>
-      </c>
+        <v>488</v>
+      </c>
+      <c r="N64" s="2"/>
+      <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
         <v>18</v>
       </c>
@@ -9760,13 +9794,13 @@
         <v>18</v>
       </c>
       <c r="X64" t="s" s="2">
-        <v>154</v>
+        <v>18</v>
       </c>
       <c r="Y64" t="s" s="2">
-        <v>494</v>
+        <v>18</v>
       </c>
       <c r="Z64" t="s" s="2">
-        <v>495</v>
+        <v>18</v>
       </c>
       <c r="AA64" t="s" s="2">
         <v>18</v>
@@ -9784,16 +9818,16 @@
         <v>18</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH64" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI64" t="s" s="2">
-        <v>18</v>
+        <v>483</v>
       </c>
       <c r="AJ64" t="s" s="2">
         <v>100</v>
@@ -9802,13 +9836,13 @@
         <v>18</v>
       </c>
       <c r="AL64" t="s" s="2">
-        <v>487</v>
+        <v>18</v>
       </c>
       <c r="AM64" t="s" s="2">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="AN64" t="s" s="2">
-        <v>406</v>
+        <v>489</v>
       </c>
       <c r="AO64" t="s" s="2">
         <v>18</v>
@@ -9819,10 +9853,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9845,17 +9879,19 @@
         <v>18</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>497</v>
+        <v>236</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>499</v>
-      </c>
-      <c r="N65" s="2"/>
+        <v>492</v>
+      </c>
+      <c r="N65" t="s" s="2">
+        <v>493</v>
+      </c>
       <c r="O65" t="s" s="2">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="P65" t="s" s="2">
         <v>18</v>
@@ -9880,13 +9916,13 @@
         <v>18</v>
       </c>
       <c r="X65" t="s" s="2">
-        <v>18</v>
+        <v>168</v>
       </c>
       <c r="Y65" t="s" s="2">
-        <v>18</v>
+        <v>495</v>
       </c>
       <c r="Z65" t="s" s="2">
-        <v>18</v>
+        <v>496</v>
       </c>
       <c r="AA65" t="s" s="2">
         <v>18</v>
@@ -9904,7 +9940,7 @@
         <v>18</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>76</v>
@@ -9922,13 +9958,13 @@
         <v>18</v>
       </c>
       <c r="AL65" t="s" s="2">
-        <v>18</v>
+        <v>497</v>
       </c>
       <c r="AM65" t="s" s="2">
-        <v>18</v>
+        <v>498</v>
       </c>
       <c r="AN65" t="s" s="2">
-        <v>501</v>
+        <v>416</v>
       </c>
       <c r="AO65" t="s" s="2">
         <v>18</v>
@@ -9939,10 +9975,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -9953,7 +9989,7 @@
         <v>76</v>
       </c>
       <c r="G66" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H66" t="s" s="2">
         <v>18</v>
@@ -9965,16 +10001,20 @@
         <v>18</v>
       </c>
       <c r="K66" t="s" s="2">
-        <v>102</v>
+        <v>236</v>
       </c>
       <c r="L66" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="M66" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="N66" t="s" s="2">
+        <v>502</v>
+      </c>
+      <c r="O66" t="s" s="2">
         <v>503</v>
       </c>
-      <c r="M66" t="s" s="2">
-        <v>504</v>
-      </c>
-      <c r="N66" s="2"/>
-      <c r="O66" s="2"/>
       <c r="P66" t="s" s="2">
         <v>18</v>
       </c>
@@ -9998,13 +10038,13 @@
         <v>18</v>
       </c>
       <c r="X66" t="s" s="2">
-        <v>18</v>
+        <v>154</v>
       </c>
       <c r="Y66" t="s" s="2">
-        <v>18</v>
+        <v>504</v>
       </c>
       <c r="Z66" t="s" s="2">
-        <v>18</v>
+        <v>505</v>
       </c>
       <c r="AA66" t="s" s="2">
         <v>18</v>
@@ -10022,13 +10062,13 @@
         <v>18</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH66" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI66" t="s" s="2">
         <v>18</v>
@@ -10040,13 +10080,13 @@
         <v>18</v>
       </c>
       <c r="AL66" t="s" s="2">
-        <v>18</v>
+        <v>497</v>
       </c>
       <c r="AM66" t="s" s="2">
-        <v>474</v>
+        <v>498</v>
       </c>
       <c r="AN66" t="s" s="2">
-        <v>505</v>
+        <v>416</v>
       </c>
       <c r="AO66" t="s" s="2">
         <v>18</v>
@@ -10071,7 +10111,7 @@
         <v>76</v>
       </c>
       <c r="G67" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H67" t="s" s="2">
         <v>18</v>
@@ -10080,7 +10120,7 @@
         <v>18</v>
       </c>
       <c r="J67" t="s" s="2">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="K67" t="s" s="2">
         <v>507</v>
@@ -10091,10 +10131,10 @@
       <c r="M67" t="s" s="2">
         <v>509</v>
       </c>
-      <c r="N67" t="s" s="2">
+      <c r="N67" s="2"/>
+      <c r="O67" t="s" s="2">
         <v>510</v>
       </c>
-      <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
         <v>18</v>
       </c>
@@ -10148,7 +10188,7 @@
         <v>76</v>
       </c>
       <c r="AH67" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI67" t="s" s="2">
         <v>18</v>
@@ -10163,10 +10203,10 @@
         <v>18</v>
       </c>
       <c r="AM67" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AN67" t="s" s="2">
         <v>511</v>
-      </c>
-      <c r="AN67" t="s" s="2">
-        <v>512</v>
       </c>
       <c r="AO67" t="s" s="2">
         <v>18</v>
@@ -10177,10 +10217,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -10191,7 +10231,7 @@
         <v>76</v>
       </c>
       <c r="G68" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H68" t="s" s="2">
         <v>18</v>
@@ -10200,20 +10240,18 @@
         <v>18</v>
       </c>
       <c r="J68" t="s" s="2">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="K68" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="L68" t="s" s="2">
+        <v>513</v>
+      </c>
+      <c r="M68" t="s" s="2">
         <v>514</v>
       </c>
-      <c r="L68" t="s" s="2">
-        <v>515</v>
-      </c>
-      <c r="M68" t="s" s="2">
-        <v>516</v>
-      </c>
-      <c r="N68" t="s" s="2">
-        <v>517</v>
-      </c>
+      <c r="N68" s="2"/>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
         <v>18</v>
@@ -10262,13 +10300,13 @@
         <v>18</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH68" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI68" t="s" s="2">
         <v>18</v>
@@ -10283,10 +10321,10 @@
         <v>18</v>
       </c>
       <c r="AM68" t="s" s="2">
-        <v>511</v>
+        <v>484</v>
       </c>
       <c r="AN68" t="s" s="2">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="AO68" t="s" s="2">
         <v>18</v>
@@ -10297,10 +10335,10 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -10323,20 +10361,18 @@
         <v>89</v>
       </c>
       <c r="K69" t="s" s="2">
-        <v>454</v>
+        <v>517</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="M69" t="s" s="2">
+        <v>519</v>
+      </c>
+      <c r="N69" t="s" s="2">
         <v>520</v>
       </c>
-      <c r="M69" t="s" s="2">
-        <v>521</v>
-      </c>
-      <c r="N69" t="s" s="2">
-        <v>522</v>
-      </c>
-      <c r="O69" t="s" s="2">
-        <v>523</v>
-      </c>
+      <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
         <v>18</v>
       </c>
@@ -10384,7 +10420,7 @@
         <v>18</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>76</v>
@@ -10405,10 +10441,10 @@
         <v>18</v>
       </c>
       <c r="AM69" t="s" s="2">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="AN69" t="s" s="2">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="AO69" t="s" s="2">
         <v>18</v>
@@ -10419,10 +10455,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -10433,7 +10469,7 @@
         <v>76</v>
       </c>
       <c r="G70" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H70" t="s" s="2">
         <v>18</v>
@@ -10442,18 +10478,20 @@
         <v>18</v>
       </c>
       <c r="J70" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>102</v>
+        <v>524</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>103</v>
+        <v>525</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="N70" s="2"/>
+        <v>526</v>
+      </c>
+      <c r="N70" t="s" s="2">
+        <v>527</v>
+      </c>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
         <v>18</v>
@@ -10502,19 +10540,19 @@
         <v>18</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>105</v>
+        <v>523</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH70" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI70" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AJ70" t="s" s="2">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="AK70" t="s" s="2">
         <v>18</v>
@@ -10523,10 +10561,10 @@
         <v>18</v>
       </c>
       <c r="AM70" t="s" s="2">
-        <v>18</v>
+        <v>521</v>
       </c>
       <c r="AN70" t="s" s="2">
-        <v>106</v>
+        <v>528</v>
       </c>
       <c r="AO70" t="s" s="2">
         <v>18</v>
@@ -10537,14 +10575,14 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
-        <v>108</v>
+        <v>18</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" t="s" s="2">
@@ -10560,21 +10598,23 @@
         <v>18</v>
       </c>
       <c r="J71" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>109</v>
+        <v>464</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>110</v>
+        <v>530</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>111</v>
+        <v>531</v>
       </c>
       <c r="N71" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="O71" s="2"/>
+        <v>532</v>
+      </c>
+      <c r="O71" t="s" s="2">
+        <v>533</v>
+      </c>
       <c r="P71" t="s" s="2">
         <v>18</v>
       </c>
@@ -10622,7 +10662,7 @@
         <v>18</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>116</v>
+        <v>529</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>76</v>
@@ -10634,7 +10674,7 @@
         <v>18</v>
       </c>
       <c r="AJ71" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK71" t="s" s="2">
         <v>18</v>
@@ -10643,10 +10683,10 @@
         <v>18</v>
       </c>
       <c r="AM71" t="s" s="2">
-        <v>18</v>
+        <v>534</v>
       </c>
       <c r="AN71" t="s" s="2">
-        <v>106</v>
+        <v>535</v>
       </c>
       <c r="AO71" t="s" s="2">
         <v>18</v>
@@ -10657,46 +10697,42 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
-        <v>465</v>
+        <v>18</v>
       </c>
       <c r="E72" s="2"/>
       <c r="F72" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G72" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H72" t="s" s="2">
         <v>18</v>
       </c>
       <c r="I72" t="s" s="2">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="J72" t="s" s="2">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="K72" t="s" s="2">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>466</v>
+        <v>103</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="N72" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="O72" t="s" s="2">
-        <v>194</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N72" s="2"/>
+      <c r="O72" s="2"/>
       <c r="P72" t="s" s="2">
         <v>18</v>
       </c>
@@ -10744,19 +10780,19 @@
         <v>18</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>468</v>
+        <v>105</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH72" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI72" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AJ72" t="s" s="2">
-        <v>117</v>
+        <v>18</v>
       </c>
       <c r="AK72" t="s" s="2">
         <v>18</v>
@@ -10768,7 +10804,7 @@
         <v>18</v>
       </c>
       <c r="AN72" t="s" s="2">
-        <v>187</v>
+        <v>106</v>
       </c>
       <c r="AO72" t="s" s="2">
         <v>18</v>
@@ -10779,21 +10815,21 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>529</v>
+        <v>537</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>529</v>
+        <v>537</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
-        <v>18</v>
+        <v>108</v>
       </c>
       <c r="E73" s="2"/>
       <c r="F73" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="G73" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H73" t="s" s="2">
         <v>18</v>
@@ -10802,23 +10838,21 @@
         <v>18</v>
       </c>
       <c r="J73" t="s" s="2">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>236</v>
+        <v>109</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>530</v>
+        <v>110</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>531</v>
+        <v>111</v>
       </c>
       <c r="N73" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="O73" t="s" s="2">
-        <v>250</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="O73" s="2"/>
       <c r="P73" t="s" s="2">
         <v>18</v>
       </c>
@@ -10842,13 +10876,13 @@
         <v>18</v>
       </c>
       <c r="X73" t="s" s="2">
-        <v>154</v>
+        <v>18</v>
       </c>
       <c r="Y73" t="s" s="2">
-        <v>251</v>
+        <v>18</v>
       </c>
       <c r="Z73" t="s" s="2">
-        <v>252</v>
+        <v>18</v>
       </c>
       <c r="AA73" t="s" s="2">
         <v>18</v>
@@ -10866,34 +10900,34 @@
         <v>18</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>529</v>
+        <v>116</v>
       </c>
       <c r="AG73" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="AH73" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI73" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AJ73" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK73" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AL73" t="s" s="2">
-        <v>533</v>
+        <v>18</v>
       </c>
       <c r="AM73" t="s" s="2">
-        <v>255</v>
+        <v>18</v>
       </c>
       <c r="AN73" t="s" s="2">
-        <v>256</v>
+        <v>106</v>
       </c>
       <c r="AO73" t="s" s="2">
-        <v>257</v>
+        <v>18</v>
       </c>
       <c r="AP73" t="s" s="2">
         <v>18</v>
@@ -10901,45 +10935,45 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
-        <v>18</v>
+        <v>475</v>
       </c>
       <c r="E74" s="2"/>
       <c r="F74" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G74" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="H74" t="s" s="2">
         <v>18</v>
       </c>
       <c r="I74" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="J74" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K74" t="s" s="2">
-        <v>535</v>
+        <v>109</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>536</v>
+        <v>476</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>378</v>
+        <v>477</v>
       </c>
       <c r="N74" t="s" s="2">
-        <v>537</v>
+        <v>112</v>
       </c>
       <c r="O74" t="s" s="2">
-        <v>380</v>
+        <v>194</v>
       </c>
       <c r="P74" t="s" s="2">
         <v>18</v>
@@ -10988,37 +11022,37 @@
         <v>18</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>534</v>
+        <v>478</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH74" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="AI74" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AJ74" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK74" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>538</v>
+        <v>18</v>
       </c>
       <c r="AM74" t="s" s="2">
-        <v>384</v>
+        <v>18</v>
       </c>
       <c r="AN74" t="s" s="2">
-        <v>385</v>
+        <v>187</v>
       </c>
       <c r="AO74" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP74" t="s" s="2">
-        <v>386</v>
+        <v>18</v>
       </c>
     </row>
     <row r="75" hidden="true">
@@ -11034,7 +11068,7 @@
       </c>
       <c r="E75" s="2"/>
       <c r="F75" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="G75" t="s" s="2">
         <v>88</v>
@@ -11046,7 +11080,7 @@
         <v>18</v>
       </c>
       <c r="J75" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="K75" t="s" s="2">
         <v>236</v>
@@ -11061,7 +11095,7 @@
         <v>542</v>
       </c>
       <c r="O75" t="s" s="2">
-        <v>391</v>
+        <v>250</v>
       </c>
       <c r="P75" t="s" s="2">
         <v>18</v>
@@ -11086,13 +11120,13 @@
         <v>18</v>
       </c>
       <c r="X75" t="s" s="2">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="Y75" t="s" s="2">
-        <v>392</v>
+        <v>251</v>
       </c>
       <c r="Z75" t="s" s="2">
-        <v>393</v>
+        <v>252</v>
       </c>
       <c r="AA75" t="s" s="2">
         <v>18</v>
@@ -11113,13 +11147,13 @@
         <v>539</v>
       </c>
       <c r="AG75" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="AH75" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AI75" t="s" s="2">
-        <v>394</v>
+        <v>18</v>
       </c>
       <c r="AJ75" t="s" s="2">
         <v>100</v>
@@ -11128,16 +11162,16 @@
         <v>18</v>
       </c>
       <c r="AL75" t="s" s="2">
-        <v>18</v>
+        <v>543</v>
       </c>
       <c r="AM75" t="s" s="2">
-        <v>187</v>
+        <v>255</v>
       </c>
       <c r="AN75" t="s" s="2">
-        <v>395</v>
+        <v>256</v>
       </c>
       <c r="AO75" t="s" s="2">
-        <v>18</v>
+        <v>257</v>
       </c>
       <c r="AP75" t="s" s="2">
         <v>18</v>
@@ -11145,21 +11179,21 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
-        <v>397</v>
+        <v>18</v>
       </c>
       <c r="E76" s="2"/>
       <c r="F76" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G76" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H76" t="s" s="2">
         <v>18</v>
@@ -11168,22 +11202,22 @@
         <v>18</v>
       </c>
       <c r="J76" t="s" s="2">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="K76" t="s" s="2">
-        <v>236</v>
+        <v>545</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>398</v>
+        <v>546</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>399</v>
+        <v>378</v>
       </c>
       <c r="N76" t="s" s="2">
-        <v>400</v>
+        <v>547</v>
       </c>
       <c r="O76" t="s" s="2">
-        <v>401</v>
+        <v>380</v>
       </c>
       <c r="P76" t="s" s="2">
         <v>18</v>
@@ -11208,13 +11242,13 @@
         <v>18</v>
       </c>
       <c r="X76" t="s" s="2">
-        <v>146</v>
+        <v>18</v>
       </c>
       <c r="Y76" t="s" s="2">
-        <v>402</v>
+        <v>18</v>
       </c>
       <c r="Z76" t="s" s="2">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="AA76" t="s" s="2">
         <v>18</v>
@@ -11232,13 +11266,13 @@
         <v>18</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH76" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI76" t="s" s="2">
         <v>18</v>
@@ -11250,27 +11284,27 @@
         <v>18</v>
       </c>
       <c r="AL76" t="s" s="2">
-        <v>404</v>
+        <v>548</v>
       </c>
       <c r="AM76" t="s" s="2">
-        <v>405</v>
+        <v>385</v>
       </c>
       <c r="AN76" t="s" s="2">
-        <v>406</v>
+        <v>386</v>
       </c>
       <c r="AO76" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP76" t="s" s="2">
-        <v>407</v>
+        <v>387</v>
       </c>
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -11281,7 +11315,7 @@
         <v>76</v>
       </c>
       <c r="G77" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="H77" t="s" s="2">
         <v>18</v>
@@ -11293,19 +11327,19 @@
         <v>18</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>18</v>
+        <v>236</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="N77" t="s" s="2">
-        <v>457</v>
+        <v>552</v>
       </c>
       <c r="O77" t="s" s="2">
-        <v>458</v>
+        <v>401</v>
       </c>
       <c r="P77" t="s" s="2">
         <v>18</v>
@@ -11330,13 +11364,13 @@
         <v>18</v>
       </c>
       <c r="X77" t="s" s="2">
-        <v>18</v>
+        <v>146</v>
       </c>
       <c r="Y77" t="s" s="2">
-        <v>18</v>
+        <v>402</v>
       </c>
       <c r="Z77" t="s" s="2">
-        <v>18</v>
+        <v>403</v>
       </c>
       <c r="AA77" t="s" s="2">
         <v>18</v>
@@ -11354,16 +11388,16 @@
         <v>18</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AH77" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="AI77" t="s" s="2">
-        <v>18</v>
+        <v>404</v>
       </c>
       <c r="AJ77" t="s" s="2">
         <v>100</v>
@@ -11375,20 +11409,264 @@
         <v>18</v>
       </c>
       <c r="AM77" t="s" s="2">
-        <v>460</v>
+        <v>187</v>
       </c>
       <c r="AN77" t="s" s="2">
-        <v>461</v>
+        <v>405</v>
       </c>
       <c r="AO77" t="s" s="2">
         <v>18</v>
       </c>
       <c r="AP77" t="s" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="78" hidden="true">
+      <c r="A78" t="s" s="2">
+        <v>553</v>
+      </c>
+      <c r="B78" t="s" s="2">
+        <v>553</v>
+      </c>
+      <c r="C78" s="2"/>
+      <c r="D78" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="E78" s="2"/>
+      <c r="F78" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G78" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="I78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="K78" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="L78" t="s" s="2">
+        <v>408</v>
+      </c>
+      <c r="M78" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="N78" t="s" s="2">
+        <v>410</v>
+      </c>
+      <c r="O78" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="P78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="Q78" s="2"/>
+      <c r="R78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="S78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="T78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="U78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="V78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="W78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="X78" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="Y78" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="Z78" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="AA78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AB78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AC78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AD78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AE78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AF78" t="s" s="2">
+        <v>553</v>
+      </c>
+      <c r="AG78" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH78" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AJ78" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AL78" t="s" s="2">
+        <v>414</v>
+      </c>
+      <c r="AM78" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="AN78" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="AO78" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AP78" t="s" s="2">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="79" hidden="true">
+      <c r="A79" t="s" s="2">
+        <v>554</v>
+      </c>
+      <c r="B79" t="s" s="2">
+        <v>554</v>
+      </c>
+      <c r="C79" s="2"/>
+      <c r="D79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="E79" s="2"/>
+      <c r="F79" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="G79" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="I79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="K79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="L79" t="s" s="2">
+        <v>555</v>
+      </c>
+      <c r="M79" t="s" s="2">
+        <v>556</v>
+      </c>
+      <c r="N79" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="O79" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="P79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="Q79" s="2"/>
+      <c r="R79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="S79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="T79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="U79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="V79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="W79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="X79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="Y79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="Z79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AA79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AB79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AC79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AD79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AE79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AF79" t="s" s="2">
+        <v>554</v>
+      </c>
+      <c r="AG79" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AH79" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AI79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AJ79" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AK79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AL79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AM79" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="AN79" t="s" s="2">
+        <v>471</v>
+      </c>
+      <c r="AO79" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="AP79" t="s" s="2">
         <v>18</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP77">
+  <autoFilter ref="A1:AP79">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -11398,7 +11676,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI76">
+  <conditionalFormatting sqref="A2:AI78">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>